<commit_message>
✅ Hoàn thành Phase A: Củng cố deterministic engine
</commit_message>
<xml_diff>
--- a/product Tester/templates/test-cases.xlsx
+++ b/product Tester/templates/test-cases.xlsx
@@ -53,7 +53,8 @@
     <t>Verify that the website link is accessible</t>
   </si>
   <si>
-    <t>1. Open browser 2. Navigate to http://localhost:3000</t>
+    <t>1. Open browser 
+2. Navigate to http://localhost:3000</t>
   </si>
   <si>
     <t>The website interface is fully loaded and displayed correctly</t>
@@ -68,7 +69,10 @@
     <t>Verify that a user can login with valid credentials</t>
   </si>
   <si>
-    <t>1. Go to Login page 2. Enter username: "ctn" 3. Enter password: "12345678" 4. Click Login button</t>
+    <t>1. Go to Login page 
+2. Enter username: "ctn" 
+3. Enter password: "12345678" 
+4. Click Login button</t>
   </si>
   <si>
     <t>User is successfully redirected to the dashboard</t>
@@ -83,7 +87,11 @@
     <t>Verify that a user can register a new account</t>
   </si>
   <si>
-    <t>1. Click Register button 2. Enter username: "tester11" 3. Enter email: "tester11@gmail.com" 4. Enter password: "12345678" 5. Click Submit</t>
+    <t>1. Click Register button 
+2. Enter username: "tester112" 
+3. Enter email: "tester112@gmail.com" 
+4. Enter password: "123456789" 
+5. Click Submit</t>
   </si>
   <si>
     <t>Registration is successful and user is redirected to the Login page</t>
@@ -113,7 +121,9 @@
     <t>Verify the "Forgot Password" functionality</t>
   </si>
   <si>
-    <t>1. Click "Forgot Password" 2. Enter email used in TC-033. Click "Send Reset Link"</t>
+    <t>1. Click "Forgot Password" 
+2. Enter email used in TC-03
+3. Click "Send Reset Link"</t>
   </si>
   <si>
     <t>System displays: "Reset link sent to email (check console)"</t>
@@ -1197,7 +1207,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" ht="40.35" spans="1:5">
+    <row r="3" ht="53.55" spans="1:5">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1214,7 +1224,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" ht="66.75" spans="1:5">
+    <row r="4" ht="79.95" spans="1:5">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
docs(root): add root README for better project presentation
</commit_message>
<xml_diff>
--- a/product Tester/templates/test-cases.xlsx
+++ b/product Tester/templates/test-cases.xlsx
@@ -27,106 +27,180 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="58">
   <si>
     <t>ID</t>
   </si>
   <si>
+    <t>Category</t>
+  </si>
+  <si>
     <t>Scenario</t>
   </si>
   <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Steps</t>
-  </si>
-  <si>
     <t>Expected Result</t>
   </si>
   <si>
     <t>TC-01</t>
   </si>
   <si>
-    <t>Check Link</t>
-  </si>
-  <si>
-    <t>Verify that the website link is accessible</t>
-  </si>
-  <si>
-    <t>1. Open browser 
-2. Navigate to http://localhost:3000</t>
-  </si>
-  <si>
-    <t>The website interface is fully loaded and displayed correctly</t>
+    <t>UI</t>
+  </si>
+  <si>
+    <t>Kiểm tra font chữ và màu sắc</t>
+  </si>
+  <si>
+    <t>Font chữ đồng nhất, dễ đọc, không bị lỗi mã hóa tiếng Việt</t>
   </si>
   <si>
     <t>TC-02</t>
   </si>
   <si>
-    <t>User Login</t>
-  </si>
-  <si>
-    <t>Verify that a user can login with valid credentials</t>
-  </si>
-  <si>
-    <t>1. Go to Login page 
-2. Enter username: "ctn" 
-3. Enter password: "12345678" 
-4. Click Login button</t>
-  </si>
-  <si>
-    <t>User is successfully redirected to the dashboard</t>
+    <t>Kiểm tra ảnh đại diện (Avatar)</t>
+  </si>
+  <si>
+    <t>Ảnh hiển thị rõ nét, không bị méo hoặc vỡ hình</t>
   </si>
   <si>
     <t>TC-03</t>
   </si>
   <si>
-    <t>User Registration</t>
-  </si>
-  <si>
-    <t>Verify that a user can register a new account</t>
-  </si>
-  <si>
-    <t>1. Click Register button 
-2. Enter username: "tester112" 
-3. Enter email: "tester112@gmail.com" 
-4. Enter password: "123456789" 
-5. Click Submit</t>
-  </si>
-  <si>
-    <t>Registration is successful and user is redirected to the Login page</t>
+    <t>Content</t>
+  </si>
+  <si>
+    <t>Kiểm tra thông tin giới thiệu</t>
+  </si>
+  <si>
+    <t>Thông tin tiểu sử hiển thị đầy đủ, không có lỗi chính tả</t>
   </si>
   <si>
     <t>TC-04</t>
   </si>
   <si>
-    <t>User Logout</t>
-  </si>
-  <si>
-    <t>Verify that a user can logout from the system</t>
-  </si>
-  <si>
-    <t>1. Login with credentials from TC-03 2. Click Logout button</t>
-  </si>
-  <si>
-    <t>User is logged out and redirected back to the landing page</t>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>Kiểm tra thanh Menu/Navigation</t>
+  </si>
+  <si>
+    <t>Click các mục trên menu chuyển đúng đến phần tương ứng trên trang</t>
   </si>
   <si>
     <t>TC-05</t>
   </si>
   <si>
-    <t>Forgot Password</t>
-  </si>
-  <si>
-    <t>Verify the "Forgot Password" functionality</t>
-  </si>
-  <si>
-    <t>1. Click "Forgot Password" 
-2. Enter email used in TC-03
-3. Click "Send Reset Link"</t>
-  </si>
-  <si>
-    <t>System displays: "Reset link sent to email (check console)"</t>
+    <t>Kiểm tra hiệu ứng Hover</t>
+  </si>
+  <si>
+    <t>Các nút hoặc link đổi màu/hiệu ứng khi di chuột vào</t>
+  </si>
+  <si>
+    <t>TC-06</t>
+  </si>
+  <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>Kiểm tra nút "Back to top"</t>
+  </si>
+  <si>
+    <t>Khi cuộn xuống dưới, nút xuất hiện và click sẽ đưa lên đầu trang</t>
+  </si>
+  <si>
+    <t>TC-07</t>
+  </si>
+  <si>
+    <t>Project</t>
+  </si>
+  <si>
+    <t>Kiểm tra ảnh minh họa dự án</t>
+  </si>
+  <si>
+    <t>Tất cả ảnh dự án đều tải được, không bị dấu X đỏ</t>
+  </si>
+  <si>
+    <t>TC-08</t>
+  </si>
+  <si>
+    <t>Social</t>
+  </si>
+  <si>
+    <t>Kiểm tra link Facebook</t>
+  </si>
+  <si>
+    <t>Link dẫn đến đúng Profile, không bị chết link</t>
+  </si>
+  <si>
+    <t>TC-09</t>
+  </si>
+  <si>
+    <t>Kiểm tra link GitHub</t>
+  </si>
+  <si>
+    <t>Link dẫn đến đúng danh sách repository của chủ web</t>
+  </si>
+  <si>
+    <t>TC-10</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>Kiểm tra tốc độ tải trang</t>
+  </si>
+  <si>
+    <t>Trang tải hoàn tất trong dưới 3 giây với tốc độ mạng thường</t>
+  </si>
+  <si>
+    <t>TC-11</t>
+  </si>
+  <si>
+    <t>Cross-Browser</t>
+  </si>
+  <si>
+    <t>Kiểm tra trên Chrome/Firefox/Safari</t>
+  </si>
+  <si>
+    <t>Web hoạt động ổn định và hiển thị giống nhau trên các trình duyệt</t>
+  </si>
+  <si>
+    <t>TC-12</t>
+  </si>
+  <si>
+    <t>Kiểm tra mô tả dự án</t>
+  </si>
+  <si>
+    <t>Mỗi dự án đều có tên và mô tả công nghệ sử dụng rõ ràng</t>
+  </si>
+  <si>
+    <t>TC-13</t>
+  </si>
+  <si>
+    <t>Kiểm tra link tải CV (nếu có)</t>
+  </si>
+  <si>
+    <t>Click nút "Download CV" phải tải về đúng file PDF</t>
+  </si>
+  <si>
+    <t>TC-14</t>
+  </si>
+  <si>
+    <t>SEO</t>
+  </si>
+  <si>
+    <t>Kiểm tra tiêu đề trang (Title)</t>
+  </si>
+  <si>
+    <t>Tab trình duyệt hiển thị đúng tên chủ sở hữu web "Chu Thân Nhất"</t>
+  </si>
+  <si>
+    <t>TC-15</t>
+  </si>
+  <si>
+    <t>Kiểm tra khoảng cách (Spacing)</t>
+  </si>
+  <si>
+    <t>Các khối nội dung không bị dính sát vào nhau hoặc quá xa</t>
   </si>
 </sst>
 </file>
@@ -139,13 +213,20 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.5"/>
+      <color rgb="FF0A0A0A"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
@@ -154,6 +235,12 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="10.5"/>
+      <color rgb="FF0A0A0A"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -305,7 +392,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -314,6 +401,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -499,12 +592,21 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFDCDFE5"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -623,28 +725,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -653,133 +746,157 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment/>
       <extLst>
         <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
           <etc:displayText val="2"/>
         </ext>
       </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1164,11 +1281,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6" outlineLevelRow="5" outlineLevelCol="4"/>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="14.5" customWidth="1"/>
-    <col min="2" max="4" width="27.3" customWidth="1"/>
+    <col min="2" max="3" width="27.3" customWidth="1"/>
+    <col min="4" max="4" width="45.9" customWidth="1"/>
     <col min="5" max="5" width="55.6" customWidth="1"/>
     <col min="6" max="6" width="27.3" customWidth="1"/>
   </cols>
@@ -1186,93 +1304,221 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" ht="28.35" spans="1:5">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="B2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="5"/>
     </row>
-    <row r="2" ht="27.15" spans="1:5">
-      <c r="A2" s="1" t="s">
+    <row r="3" ht="28.35" spans="1:5">
+      <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
+      <c r="D3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="5"/>
     </row>
-    <row r="3" ht="53.55" spans="1:5">
-      <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="1" t="s">
+    <row r="4" ht="28.35" spans="1:5">
+      <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="B4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="C4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="D4" s="4" t="s">
         <v>14</v>
       </c>
+      <c r="E4" s="5"/>
     </row>
-    <row r="4" ht="79.95" spans="1:5">
-      <c r="A4" s="1" t="s">
+    <row r="5" ht="42.15" spans="1:5">
+      <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E5" s="5"/>
+    </row>
+    <row r="6" ht="28.35" spans="1:5">
+      <c r="A6" s="3" t="s">
         <v>19</v>
       </c>
+      <c r="B6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="5"/>
     </row>
-    <row r="5" ht="27.15" spans="1:5">
-      <c r="A5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="1" t="s">
+    <row r="7" ht="42.15" spans="1:4">
+      <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="B7" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="D7" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="6" ht="40.35" spans="1:5">
-      <c r="A6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="1" t="s">
+    <row r="8" ht="28.35" spans="1:4">
+      <c r="A8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="B8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="C8" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="D8" s="4" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="9" ht="28.35" spans="1:4">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" ht="28.35" spans="1:4">
+      <c r="A10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" ht="28.35" spans="1:4">
+      <c r="A11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" ht="42.15" spans="1:4">
+      <c r="A12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" ht="28.35" spans="1:4">
+      <c r="A13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" ht="28.35" spans="1:4">
+      <c r="A15" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" ht="27.6" spans="1:4">
+      <c r="A16" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(product-tester): improve runner, executor, and assertion logic with better reliability
</commit_message>
<xml_diff>
--- a/product Tester/templates/test-cases.xlsx
+++ b/product Tester/templates/test-cases.xlsx
@@ -27,180 +27,107 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>ID</t>
   </si>
   <si>
-    <t>Category</t>
-  </si>
-  <si>
     <t>Scenario</t>
   </si>
   <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Steps</t>
+  </si>
+  <si>
     <t>Expected Result</t>
   </si>
   <si>
     <t>TC-01</t>
   </si>
   <si>
-    <t>UI</t>
-  </si>
-  <si>
-    <t>Kiểm tra font chữ và màu sắc</t>
-  </si>
-  <si>
-    <t>Font chữ đồng nhất, dễ đọc, không bị lỗi mã hóa tiếng Việt</t>
+    <t>Check Link</t>
+  </si>
+  <si>
+    <t>Verify that the website link is accessible</t>
+  </si>
+  <si>
+    <t>1. Open browser
+2. Navigate to http://localhost:3000</t>
+  </si>
+  <si>
+    <t>The website interface is fully loaded and displayed correctly</t>
   </si>
   <si>
     <t>TC-02</t>
   </si>
   <si>
-    <t>Kiểm tra ảnh đại diện (Avatar)</t>
-  </si>
-  <si>
-    <t>Ảnh hiển thị rõ nét, không bị méo hoặc vỡ hình</t>
+    <t>User Login</t>
+  </si>
+  <si>
+    <t>Verify that a user can login with valid credentials</t>
+  </si>
+  <si>
+    <t>1. Go to Login page
+2. Enter username: "ctn"
+3. Enter password: "12345678"
+4. Click Login button</t>
+  </si>
+  <si>
+    <t>User is successfully redirected to the dashboard</t>
   </si>
   <si>
     <t>TC-03</t>
   </si>
   <si>
-    <t>Content</t>
-  </si>
-  <si>
-    <t>Kiểm tra thông tin giới thiệu</t>
-  </si>
-  <si>
-    <t>Thông tin tiểu sử hiển thị đầy đủ, không có lỗi chính tả</t>
+    <t>User Registration</t>
+  </si>
+  <si>
+    <t>Verify that a user can register a new account</t>
+  </si>
+  <si>
+    <t>1. Click Register button
+2. Enter username: "tester112"
+3. Enter email: "tester112@gmail.com"
+4. Enter password: "123456789"
+5. Click Submit</t>
+  </si>
+  <si>
+    <t>Registration is successful and user is redirected to the Login page</t>
   </si>
   <si>
     <t>TC-04</t>
   </si>
   <si>
-    <t>Function</t>
-  </si>
-  <si>
-    <t>Kiểm tra thanh Menu/Navigation</t>
-  </si>
-  <si>
-    <t>Click các mục trên menu chuyển đúng đến phần tương ứng trên trang</t>
+    <t>User Logout</t>
+  </si>
+  <si>
+    <t>Verify that a user can logout from the system</t>
+  </si>
+  <si>
+    <t>1. Login with credentials from TC-03
+2. Click Logout button</t>
+  </si>
+  <si>
+    <t>User is logged out and redirected back to the landing page</t>
   </si>
   <si>
     <t>TC-05</t>
   </si>
   <si>
-    <t>Kiểm tra hiệu ứng Hover</t>
-  </si>
-  <si>
-    <t>Các nút hoặc link đổi màu/hiệu ứng khi di chuột vào</t>
-  </si>
-  <si>
-    <t>TC-06</t>
-  </si>
-  <si>
-    <t>Navigation</t>
-  </si>
-  <si>
-    <t>Kiểm tra nút "Back to top"</t>
-  </si>
-  <si>
-    <t>Khi cuộn xuống dưới, nút xuất hiện và click sẽ đưa lên đầu trang</t>
-  </si>
-  <si>
-    <t>TC-07</t>
-  </si>
-  <si>
-    <t>Project</t>
-  </si>
-  <si>
-    <t>Kiểm tra ảnh minh họa dự án</t>
-  </si>
-  <si>
-    <t>Tất cả ảnh dự án đều tải được, không bị dấu X đỏ</t>
-  </si>
-  <si>
-    <t>TC-08</t>
-  </si>
-  <si>
-    <t>Social</t>
-  </si>
-  <si>
-    <t>Kiểm tra link Facebook</t>
-  </si>
-  <si>
-    <t>Link dẫn đến đúng Profile, không bị chết link</t>
-  </si>
-  <si>
-    <t>TC-09</t>
-  </si>
-  <si>
-    <t>Kiểm tra link GitHub</t>
-  </si>
-  <si>
-    <t>Link dẫn đến đúng danh sách repository của chủ web</t>
-  </si>
-  <si>
-    <t>TC-10</t>
-  </si>
-  <si>
-    <t>Performance</t>
-  </si>
-  <si>
-    <t>Kiểm tra tốc độ tải trang</t>
-  </si>
-  <si>
-    <t>Trang tải hoàn tất trong dưới 3 giây với tốc độ mạng thường</t>
-  </si>
-  <si>
-    <t>TC-11</t>
-  </si>
-  <si>
-    <t>Cross-Browser</t>
-  </si>
-  <si>
-    <t>Kiểm tra trên Chrome/Firefox/Safari</t>
-  </si>
-  <si>
-    <t>Web hoạt động ổn định và hiển thị giống nhau trên các trình duyệt</t>
-  </si>
-  <si>
-    <t>TC-12</t>
-  </si>
-  <si>
-    <t>Kiểm tra mô tả dự án</t>
-  </si>
-  <si>
-    <t>Mỗi dự án đều có tên và mô tả công nghệ sử dụng rõ ràng</t>
-  </si>
-  <si>
-    <t>TC-13</t>
-  </si>
-  <si>
-    <t>Kiểm tra link tải CV (nếu có)</t>
-  </si>
-  <si>
-    <t>Click nút "Download CV" phải tải về đúng file PDF</t>
-  </si>
-  <si>
-    <t>TC-14</t>
-  </si>
-  <si>
-    <t>SEO</t>
-  </si>
-  <si>
-    <t>Kiểm tra tiêu đề trang (Title)</t>
-  </si>
-  <si>
-    <t>Tab trình duyệt hiển thị đúng tên chủ sở hữu web "Chu Thân Nhất"</t>
-  </si>
-  <si>
-    <t>TC-15</t>
-  </si>
-  <si>
-    <t>Kiểm tra khoảng cách (Spacing)</t>
-  </si>
-  <si>
-    <t>Các khối nội dung không bị dính sát vào nhau hoặc quá xa</t>
+    <t>Forgot Password</t>
+  </si>
+  <si>
+    <t>Verify the "Forgot Password" functionality</t>
+  </si>
+  <si>
+    <t>1. Click "Forgot Password"
+2. Enter email used in TC-03
+3. Click "Send Reset Link"</t>
+  </si>
+  <si>
+    <t>System displays: "Reset link sent to email (check console)"</t>
   </si>
 </sst>
 </file>
@@ -213,7 +140,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -229,12 +156,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="10.5"/>
       <color rgb="FF0A0A0A"/>
       <name val="Arial"/>
@@ -592,7 +513,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -601,27 +522,55 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FFDCDFE5"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
+      <left style="thin">
+        <color auto="1"/>
       </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
+      <right style="thin">
+        <color auto="1"/>
       </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
+      <top style="thin">
+        <color auto="1"/>
       </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -725,177 +674,169 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1281,7 +1222,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="14.5" customWidth="1"/>
@@ -1291,7 +1232,7 @@
     <col min="6" max="6" width="27.3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.35" spans="1:5">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1304,224 +1245,200 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" ht="28.35" spans="1:5">
-      <c r="A2" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4" t="s">
+    </row>
+    <row r="2" ht="18.6" customHeight="1" spans="1:5">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
+      </c>
       <c r="D2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" ht="28.35" spans="1:5">
-      <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="4" t="s">
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="3"/>
+    </row>
+    <row r="4" ht="29.85" customHeight="1" spans="1:5">
+      <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="5"/>
-    </row>
-    <row r="4" ht="28.35" spans="1:5">
-      <c r="A4" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="5"/>
-    </row>
-    <row r="5" ht="42.15" spans="1:5">
-      <c r="A5" s="3" t="s">
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="2"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="3"/>
+    </row>
+    <row r="6" ht="29.1" customHeight="1" spans="1:5">
+      <c r="A6" s="2"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="3"/>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="2"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="3"/>
+    </row>
+    <row r="8" ht="17.85" customHeight="1" spans="1:5">
+      <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="5"/>
-    </row>
-    <row r="6" ht="28.35" spans="1:5">
-      <c r="A6" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="4" t="s">
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="2"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" ht="27.6" customHeight="1" spans="1:5">
+      <c r="A10" s="2"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="3"/>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="2"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="3"/>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="2"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="3"/>
+    </row>
+    <row r="13" ht="17.1" customHeight="1" spans="1:5">
+      <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="5"/>
-    </row>
-    <row r="7" ht="42.15" spans="1:4">
-      <c r="A7" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="E13" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="4" t="s">
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="2"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" customHeight="1" spans="1:5">
+      <c r="A15" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="8" ht="28.35" spans="1:4">
-      <c r="A8" s="3" t="s">
+      <c r="B15" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D15" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E15" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" ht="28.35" spans="1:4">
-      <c r="A9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" ht="28.35" spans="1:4">
-      <c r="A10" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" ht="28.35" spans="1:4">
-      <c r="A11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" ht="42.15" spans="1:4">
-      <c r="A12" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" ht="28.35" spans="1:4">
-      <c r="A13" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" ht="28.35" spans="1:4">
-      <c r="A15" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="16" ht="27.6" spans="1:4">
-      <c r="A16" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>57</v>
-      </c>
+    <row r="16" spans="1:5">
+      <c r="A16" s="2"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="2"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="3"/>
     </row>
   </sheetData>
+  <mergeCells count="25">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="C8:C12"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="C15:C17"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:D7"/>
+    <mergeCell ref="D8:D12"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="D15:D17"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E7"/>
+    <mergeCell ref="E8:E12"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="E15:E17"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>